<commit_message>
Dane z autobusami + analiza SAW
</commit_message>
<xml_diff>
--- a/autobusy.xlsx
+++ b/autobusy.xlsx
@@ -5,16 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\teste\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\teste\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8B7AE24-F265-4144-98D2-846CA5BFCF34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7B6CF2B-388F-4410-B130-D259FB8112F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{78F6C6CF-C9FD-4C30-A6D3-8F4A203AF3AD}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{78F6C6CF-C9FD-4C30-A6D3-8F4A203AF3AD}"/>
   </bookViews>
   <sheets>
     <sheet name="Duże autobusy" sheetId="1" r:id="rId1"/>
     <sheet name="Średnie autobusy" sheetId="2" r:id="rId2"/>
+    <sheet name="Duże autobusy (2)" sheetId="3" r:id="rId3"/>
+    <sheet name="Średnie autobusy (2)" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,14 +35,14 @@
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="2"/>
+      <xlwcv:version warnBelowVersion="2" setVersion="2"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="50">
   <si>
     <t>Model</t>
   </si>
@@ -163,14 +165,42 @@
   </si>
   <si>
     <t>rampa, miejsce na wózek, przyklęk</t>
+  </si>
+  <si>
+    <t>moc silnika [KM] MAX</t>
+  </si>
+  <si>
+    <t>miejsca dla pasażerów MAX</t>
+  </si>
+  <si>
+    <t>udogodnienia dla niepełnosprawnych MAX</t>
+  </si>
+  <si>
+    <t>koszt zakupu [mln zł] MIN</t>
+  </si>
+  <si>
+    <t>prestiż MAX</t>
+  </si>
+  <si>
+    <t>MAX/MIN</t>
+  </si>
+  <si>
+    <t>koszt zakupu</t>
+  </si>
+  <si>
+    <t>SAW</t>
+  </si>
+  <si>
+    <t>Waga</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;zł&quot;;[Red]\-#,##0.00\ &quot;zł&quot;"/>
+    <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -190,7 +220,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -209,6 +239,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -222,18 +258,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -568,51 +608,51 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1AF22A7-6802-42EA-9523-249B4C0BB3CA}">
-  <dimension ref="A1:I18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="21.28515625" customWidth="1"/>
-    <col min="6" max="6" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.28515625" customWidth="1"/>
-    <col min="9" max="9" width="10.85546875" customWidth="1"/>
+    <col min="1" max="1" width="23.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.26953125" customWidth="1"/>
+    <col min="6" max="6" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.26953125" customWidth="1"/>
+    <col min="9" max="9" width="10.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>31</v>
       </c>
       <c r="G1" s="1"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -625,16 +665,16 @@
       <c r="D3" t="s">
         <v>34</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3">
         <v>2.2000000000000002</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="7">
         <f>AVERAGE(10,6,5)</f>
         <v>7</v>
       </c>
       <c r="I3" s="2"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -650,11 +690,11 @@
       <c r="E4">
         <v>2.4</v>
       </c>
-      <c r="F4" s="9">
+      <c r="F4" s="7">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>6</v>
       </c>
@@ -670,12 +710,12 @@
       <c r="E5">
         <v>1.8</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="7">
         <f>AVERAGE(5,4,10)</f>
         <v>6.333333333333333</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -691,13 +731,13 @@
       <c r="E6">
         <v>1</v>
       </c>
-      <c r="F6" s="9">
+      <c r="F6" s="7">
         <f>AVERAGE(8,8,10)</f>
         <v>8.6666666666666661</v>
       </c>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>8</v>
       </c>
@@ -713,22 +753,22 @@
       <c r="E7">
         <v>1.1000000000000001</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="7">
         <f>AVERAGE(3,1,10)</f>
         <v>4.666666666666667</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="10"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="8"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>26</v>
       </c>
@@ -744,12 +784,12 @@
       <c r="E9">
         <v>2.6</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="7">
         <f>AVERAGE(7,4,8)</f>
         <v>6.333333333333333</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>27</v>
       </c>
@@ -765,12 +805,12 @@
       <c r="E10">
         <v>1.8</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="7">
         <f>AVERAGE(9,4,6)</f>
         <v>6.333333333333333</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>28</v>
       </c>
@@ -786,23 +826,23 @@
       <c r="E11">
         <v>2</v>
       </c>
-      <c r="F11" s="9">
+      <c r="F11" s="7">
         <f>AVERAGE(4,4,1)</f>
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="10"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="8"/>
       <c r="I12" s="3"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -818,12 +858,12 @@
       <c r="E13">
         <v>3.25</v>
       </c>
-      <c r="F13" s="9">
+      <c r="F13" s="7">
         <f>AVERAGE(10,10,4)</f>
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -839,22 +879,22 @@
       <c r="E14">
         <v>1</v>
       </c>
-      <c r="F14" s="9">
+      <c r="F14" s="7">
         <f>AVERAGE(5,4,3)</f>
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="10"/>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
+      <c r="F15" s="8"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -870,22 +910,22 @@
       <c r="E16">
         <v>2</v>
       </c>
-      <c r="F16" s="9">
+      <c r="F16" s="7">
         <f>AVERAGE(8,9,9)</f>
         <v>8.6666666666666661</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="5" t="s">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A17" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="10"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="8"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>30</v>
       </c>
@@ -901,9 +941,15 @@
       <c r="E18">
         <v>2.9</v>
       </c>
-      <c r="F18" s="9">
+      <c r="F18" s="7">
         <f>AVERAGE(10,9,10)</f>
         <v>9.6666666666666661</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="D20">
+        <f>IF(D3="",0, LEN(D3) - LEN(SUBSTITUTE(D3,",",""))+1)</f>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -914,47 +960,47 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9963985E-3EE3-41A7-B4A2-294A43F0CA3B}">
   <dimension ref="A1:F16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
     <col min="2" max="2" width="16" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="35.140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="35.1796875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -970,12 +1016,12 @@
       <c r="E3">
         <v>2.6</v>
       </c>
-      <c r="F3" s="9">
+      <c r="F3" s="7">
         <f>AVERAGE(6,4,2)</f>
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>16</v>
       </c>
@@ -991,12 +1037,12 @@
       <c r="E4">
         <v>2.4</v>
       </c>
-      <c r="F4" s="9">
+      <c r="F4" s="7">
         <f>AVERAGE(6,8,10)</f>
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -1012,22 +1058,22 @@
       <c r="E5">
         <v>1.1000000000000001</v>
       </c>
-      <c r="F5" s="9">
+      <c r="F5" s="7">
         <f>AVERAGE(10,5,5)</f>
         <v>6.666666666666667</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
-      <c r="F6" s="10"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="8"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -1043,22 +1089,22 @@
       <c r="E7">
         <v>2.6</v>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="7">
         <f>AVERAGE(5,5,5)</f>
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="5" t="s">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="10"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="8"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1074,12 +1120,12 @@
       <c r="E9">
         <v>0.6</v>
       </c>
-      <c r="F9" s="9">
+      <c r="F9" s="7">
         <f>AVERAGE(3,6,4)</f>
         <v>4.333333333333333</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -1089,18 +1135,18 @@
       <c r="C10">
         <v>24</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" s="9" t="s">
         <v>36</v>
       </c>
       <c r="E10">
         <v>2.2000000000000002</v>
       </c>
-      <c r="F10" s="9">
+      <c r="F10" s="7">
         <f>AVERAGE(5,6,4)</f>
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -1116,22 +1162,22 @@
       <c r="E11">
         <v>0.9</v>
       </c>
-      <c r="F11" s="9">
+      <c r="F11" s="7">
         <f>AVERAGE(5,7,5)</f>
         <v>5.666666666666667</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="5" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A12" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="10"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="8"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1147,22 +1193,22 @@
       <c r="E13">
         <v>1.3</v>
       </c>
-      <c r="F13" s="9">
+      <c r="F13" s="7">
         <f>AVERAGE(9,9,7)</f>
         <v>8.3333333333333339</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A14" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="10"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="8"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>33</v>
       </c>
@@ -1178,12 +1224,12 @@
       <c r="E15">
         <v>1.1000000000000001</v>
       </c>
-      <c r="F15" s="9">
+      <c r="F15" s="7">
         <f>AVERAGE(9,7,10)</f>
         <v>8.6666666666666661</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>24</v>
       </c>
@@ -1193,15 +1239,1361 @@
       <c r="C16">
         <v>47</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="E16" s="8">
+      <c r="E16">
         <v>0.9</v>
       </c>
-      <c r="F16" s="9">
+      <c r="F16" s="7">
         <f>AVERAGE(8,3,8)</f>
         <v>6.333333333333333</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF33C538-C2CB-4E1F-B5CA-2C4D84AF0445}">
+  <dimension ref="A1:I30"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="23.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.453125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.81640625" customWidth="1"/>
+    <col min="5" max="5" width="23.36328125" customWidth="1"/>
+    <col min="6" max="6" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.26953125" customWidth="1"/>
+    <col min="9" max="9" width="10.81640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2">
+        <v>408</v>
+      </c>
+      <c r="C2">
+        <v>65</v>
+      </c>
+      <c r="D2">
+        <f>IF('Duże autobusy'!D3="",0, LEN('Duże autobusy'!D3) - LEN(SUBSTITUTE('Duże autobusy'!D3,",",""))+1)</f>
+        <v>2</v>
+      </c>
+      <c r="E2">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="F2" s="7">
+        <f>AVERAGE(10,6,5)</f>
+        <v>7</v>
+      </c>
+      <c r="I2" s="2"/>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>320</v>
+      </c>
+      <c r="C3">
+        <v>55</v>
+      </c>
+      <c r="D3">
+        <f>IF('Duże autobusy'!D4="",0, LEN('Duże autobusy'!D4) - LEN(SUBSTITUTE('Duże autobusy'!D4,",",""))+1)</f>
+        <v>3</v>
+      </c>
+      <c r="E3">
+        <v>2.4</v>
+      </c>
+      <c r="F3" s="7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>310</v>
+      </c>
+      <c r="C4">
+        <v>54</v>
+      </c>
+      <c r="D4">
+        <f>IF('Duże autobusy'!D5="",0, LEN('Duże autobusy'!D5) - LEN(SUBSTITUTE('Duże autobusy'!D5,",",""))+1)</f>
+        <v>3</v>
+      </c>
+      <c r="E4">
+        <v>1.8</v>
+      </c>
+      <c r="F4" s="7">
+        <f>AVERAGE(5,4,10)</f>
+        <v>6.333333333333333</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5">
+        <v>256</v>
+      </c>
+      <c r="C5">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <f>IF('Duże autobusy'!D6="",0, LEN('Duże autobusy'!D6) - LEN(SUBSTITUTE('Duże autobusy'!D6,",",""))+1)</f>
+        <v>3</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5" s="7">
+        <f>AVERAGE(8,8,10)</f>
+        <v>8.6666666666666661</v>
+      </c>
+      <c r="I5" s="2"/>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6">
+        <v>320</v>
+      </c>
+      <c r="C6">
+        <v>40</v>
+      </c>
+      <c r="D6">
+        <f>IF('Duże autobusy'!D7="",0, LEN('Duże autobusy'!D7) - LEN(SUBSTITUTE('Duże autobusy'!D7,",",""))+1)</f>
+        <v>3</v>
+      </c>
+      <c r="E6">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="F6" s="7">
+        <f>AVERAGE(3,1,10)</f>
+        <v>4.666666666666667</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7">
+        <v>326</v>
+      </c>
+      <c r="C7">
+        <v>44</v>
+      </c>
+      <c r="D7">
+        <f>IF('Duże autobusy'!D9="",0, LEN('Duże autobusy'!D9) - LEN(SUBSTITUTE('Duże autobusy'!D9,",",""))+1)</f>
+        <v>4</v>
+      </c>
+      <c r="E7">
+        <v>2.6</v>
+      </c>
+      <c r="F7" s="7">
+        <f>AVERAGE(7,4,8)</f>
+        <v>6.333333333333333</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8">
+        <v>265</v>
+      </c>
+      <c r="C8">
+        <v>63</v>
+      </c>
+      <c r="D8">
+        <f>IF('Duże autobusy'!D10="",0, LEN('Duże autobusy'!D10) - LEN(SUBSTITUTE('Duże autobusy'!D10,",",""))+1)</f>
+        <v>3</v>
+      </c>
+      <c r="E8">
+        <v>1.8</v>
+      </c>
+      <c r="F8" s="7">
+        <f>AVERAGE(9,4,6)</f>
+        <v>6.333333333333333</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9">
+        <v>280</v>
+      </c>
+      <c r="C9">
+        <v>37</v>
+      </c>
+      <c r="D9">
+        <f>IF('Duże autobusy'!D11="",0, LEN('Duże autobusy'!D11) - LEN(SUBSTITUTE('Duże autobusy'!D11,",",""))+1)</f>
+        <v>4</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+      <c r="F9" s="7">
+        <f>AVERAGE(4,4,1)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10">
+        <v>344</v>
+      </c>
+      <c r="C10">
+        <v>40</v>
+      </c>
+      <c r="D10">
+        <f>IF('Duże autobusy'!D13="",0, LEN('Duże autobusy'!D13) - LEN(SUBSTITUTE('Duże autobusy'!D13,",",""))+1)</f>
+        <v>3</v>
+      </c>
+      <c r="E10">
+        <v>3.25</v>
+      </c>
+      <c r="F10" s="7">
+        <f>AVERAGE(10,10,4)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11">
+        <v>277</v>
+      </c>
+      <c r="C11">
+        <v>40</v>
+      </c>
+      <c r="D11">
+        <f>IF('Duże autobusy'!D14="",0, LEN('Duże autobusy'!D14) - LEN(SUBSTITUTE('Duże autobusy'!D14,",",""))+1)</f>
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11" s="7">
+        <f>AVERAGE(5,4,3)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12">
+        <v>360</v>
+      </c>
+      <c r="C12">
+        <v>44</v>
+      </c>
+      <c r="D12">
+        <f>IF('Duże autobusy'!D16="",0, LEN('Duże autobusy'!D16) - LEN(SUBSTITUTE('Duże autobusy'!D16,",",""))+1)</f>
+        <v>4</v>
+      </c>
+      <c r="E12">
+        <v>2</v>
+      </c>
+      <c r="F12" s="7">
+        <f>AVERAGE(8,9,9)</f>
+        <v>8.6666666666666661</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13">
+        <v>340</v>
+      </c>
+      <c r="C13">
+        <v>37</v>
+      </c>
+      <c r="D13">
+        <f>IF('Duże autobusy'!D18="",0, LEN('Duże autobusy'!D18) - LEN(SUBSTITUTE('Duże autobusy'!D18,",",""))+1)</f>
+        <v>3</v>
+      </c>
+      <c r="E13">
+        <v>2.9</v>
+      </c>
+      <c r="F13" s="7">
+        <f>AVERAGE(10,9,10)</f>
+        <v>9.6666666666666661</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15">
+        <f>MAX(B2:B13)</f>
+        <v>408</v>
+      </c>
+      <c r="C15">
+        <f>MAX(C2:C13)</f>
+        <v>65</v>
+      </c>
+      <c r="D15">
+        <f>MAX(D2:D13)</f>
+        <v>4</v>
+      </c>
+      <c r="E15">
+        <f>MIN(E2:E13)</f>
+        <v>1</v>
+      </c>
+      <c r="F15">
+        <f>MAX(F2:F13)</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>49</v>
+      </c>
+      <c r="B16">
+        <v>0.26</v>
+      </c>
+      <c r="C16">
+        <v>0.26</v>
+      </c>
+      <c r="D16">
+        <v>0.11</v>
+      </c>
+      <c r="E16">
+        <v>0.11</v>
+      </c>
+      <c r="F16">
+        <v>0.26</v>
+      </c>
+      <c r="G16">
+        <f>SUM(B16:F16)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>4</v>
+      </c>
+      <c r="B19" s="11">
+        <f>(B2/B$15)*B$16</f>
+        <v>0.26</v>
+      </c>
+      <c r="C19" s="11">
+        <f t="shared" ref="C19:F19" si="0">(C2/C$15)*C$16</f>
+        <v>0.26</v>
+      </c>
+      <c r="D19" s="11">
+        <f t="shared" si="0"/>
+        <v>5.5E-2</v>
+      </c>
+      <c r="E19" s="11">
+        <f>($E$15/E2)*$E$16</f>
+        <v>4.9999999999999996E-2</v>
+      </c>
+      <c r="F19" s="11">
+        <f t="shared" si="0"/>
+        <v>0.182</v>
+      </c>
+      <c r="G19" s="10">
+        <f>SUM(B19:F19)</f>
+        <v>0.80700000000000016</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B20" s="14">
+        <f t="shared" ref="B20:F30" si="1">(B3/B$15)*B$16</f>
+        <v>0.20392156862745098</v>
+      </c>
+      <c r="C20" s="14">
+        <f t="shared" si="1"/>
+        <v>0.22</v>
+      </c>
+      <c r="D20" s="14">
+        <f t="shared" si="1"/>
+        <v>8.2500000000000004E-2</v>
+      </c>
+      <c r="E20" s="14">
+        <f t="shared" ref="E20:E30" si="2">($E$15/E3)*$E$16</f>
+        <v>4.5833333333333337E-2</v>
+      </c>
+      <c r="F20" s="14">
+        <f t="shared" si="1"/>
+        <v>0.26</v>
+      </c>
+      <c r="G20" s="12">
+        <f t="shared" ref="G20:G30" si="3">SUM(B20:F20)</f>
+        <v>0.81225490196078431</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>6</v>
+      </c>
+      <c r="B21" s="11">
+        <f t="shared" si="1"/>
+        <v>0.19754901960784313</v>
+      </c>
+      <c r="C21" s="11">
+        <f t="shared" si="1"/>
+        <v>0.21600000000000003</v>
+      </c>
+      <c r="D21" s="11">
+        <f t="shared" si="1"/>
+        <v>8.2500000000000004E-2</v>
+      </c>
+      <c r="E21" s="11">
+        <f t="shared" si="2"/>
+        <v>6.1111111111111116E-2</v>
+      </c>
+      <c r="F21" s="11">
+        <f t="shared" si="1"/>
+        <v>0.16466666666666666</v>
+      </c>
+      <c r="G21" s="10">
+        <f t="shared" si="3"/>
+        <v>0.72182679738562094</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>7</v>
+      </c>
+      <c r="B22" s="11">
+        <f t="shared" si="1"/>
+        <v>0.16313725490196079</v>
+      </c>
+      <c r="C22" s="11">
+        <f t="shared" si="1"/>
+        <v>6.4000000000000001E-2</v>
+      </c>
+      <c r="D22" s="11">
+        <f t="shared" si="1"/>
+        <v>8.2500000000000004E-2</v>
+      </c>
+      <c r="E22" s="11">
+        <f t="shared" si="2"/>
+        <v>0.11</v>
+      </c>
+      <c r="F22" s="11">
+        <f t="shared" si="1"/>
+        <v>0.22533333333333333</v>
+      </c>
+      <c r="G22" s="10">
+        <f t="shared" si="3"/>
+        <v>0.64497058823529407</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>8</v>
+      </c>
+      <c r="B23" s="11">
+        <f t="shared" si="1"/>
+        <v>0.20392156862745098</v>
+      </c>
+      <c r="C23" s="11">
+        <f t="shared" si="1"/>
+        <v>0.16</v>
+      </c>
+      <c r="D23" s="11">
+        <f t="shared" si="1"/>
+        <v>8.2500000000000004E-2</v>
+      </c>
+      <c r="E23" s="11">
+        <f t="shared" si="2"/>
+        <v>9.9999999999999992E-2</v>
+      </c>
+      <c r="F23" s="11">
+        <f t="shared" si="1"/>
+        <v>0.12133333333333333</v>
+      </c>
+      <c r="G23" s="10">
+        <f t="shared" si="3"/>
+        <v>0.66775490196078424</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" s="11">
+        <f t="shared" si="1"/>
+        <v>0.2077450980392157</v>
+      </c>
+      <c r="C24" s="11">
+        <f t="shared" si="1"/>
+        <v>0.17600000000000002</v>
+      </c>
+      <c r="D24" s="11">
+        <f t="shared" si="1"/>
+        <v>0.11</v>
+      </c>
+      <c r="E24" s="11">
+        <f t="shared" si="2"/>
+        <v>4.2307692307692303E-2</v>
+      </c>
+      <c r="F24" s="11">
+        <f t="shared" si="1"/>
+        <v>0.16466666666666666</v>
+      </c>
+      <c r="G24" s="10">
+        <f t="shared" si="3"/>
+        <v>0.70071945701357463</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="11">
+        <f t="shared" si="1"/>
+        <v>0.16887254901960785</v>
+      </c>
+      <c r="C25" s="11">
+        <f t="shared" si="1"/>
+        <v>0.252</v>
+      </c>
+      <c r="D25" s="11">
+        <f t="shared" si="1"/>
+        <v>8.2500000000000004E-2</v>
+      </c>
+      <c r="E25" s="11">
+        <f t="shared" si="2"/>
+        <v>6.1111111111111116E-2</v>
+      </c>
+      <c r="F25" s="11">
+        <f t="shared" si="1"/>
+        <v>0.16466666666666666</v>
+      </c>
+      <c r="G25" s="10">
+        <f t="shared" si="3"/>
+        <v>0.72915032679738556</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="11">
+        <f t="shared" si="1"/>
+        <v>0.17843137254901961</v>
+      </c>
+      <c r="C26" s="11">
+        <f t="shared" si="1"/>
+        <v>0.14799999999999999</v>
+      </c>
+      <c r="D26" s="11">
+        <f t="shared" si="1"/>
+        <v>0.11</v>
+      </c>
+      <c r="E26" s="11">
+        <f t="shared" si="2"/>
+        <v>5.5E-2</v>
+      </c>
+      <c r="F26" s="11">
+        <f t="shared" si="1"/>
+        <v>7.8E-2</v>
+      </c>
+      <c r="G26" s="10">
+        <f t="shared" si="3"/>
+        <v>0.56943137254901954</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
+        <v>11</v>
+      </c>
+      <c r="B27" s="11">
+        <f t="shared" si="1"/>
+        <v>0.21921568627450982</v>
+      </c>
+      <c r="C27" s="11">
+        <f t="shared" si="1"/>
+        <v>0.16</v>
+      </c>
+      <c r="D27" s="11">
+        <f t="shared" si="1"/>
+        <v>8.2500000000000004E-2</v>
+      </c>
+      <c r="E27" s="11">
+        <f t="shared" si="2"/>
+        <v>3.3846153846153845E-2</v>
+      </c>
+      <c r="F27" s="11">
+        <f t="shared" si="1"/>
+        <v>0.20800000000000002</v>
+      </c>
+      <c r="G27" s="10">
+        <f t="shared" si="3"/>
+        <v>0.70356184012066381</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
+        <v>12</v>
+      </c>
+      <c r="B28" s="11">
+        <f t="shared" si="1"/>
+        <v>0.17651960784313728</v>
+      </c>
+      <c r="C28" s="11">
+        <f t="shared" si="1"/>
+        <v>0.16</v>
+      </c>
+      <c r="D28" s="11">
+        <f t="shared" si="1"/>
+        <v>8.2500000000000004E-2</v>
+      </c>
+      <c r="E28" s="11">
+        <f t="shared" si="2"/>
+        <v>0.11</v>
+      </c>
+      <c r="F28" s="11">
+        <f t="shared" si="1"/>
+        <v>0.10400000000000001</v>
+      </c>
+      <c r="G28" s="10">
+        <f t="shared" si="3"/>
+        <v>0.63301960784313727</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
+        <v>14</v>
+      </c>
+      <c r="B29" s="11">
+        <f t="shared" si="1"/>
+        <v>0.22941176470588234</v>
+      </c>
+      <c r="C29" s="11">
+        <f t="shared" si="1"/>
+        <v>0.17600000000000002</v>
+      </c>
+      <c r="D29" s="11">
+        <f t="shared" si="1"/>
+        <v>0.11</v>
+      </c>
+      <c r="E29" s="11">
+        <f t="shared" si="2"/>
+        <v>5.5E-2</v>
+      </c>
+      <c r="F29" s="11">
+        <f t="shared" si="1"/>
+        <v>0.22533333333333333</v>
+      </c>
+      <c r="G29" s="10">
+        <f t="shared" si="3"/>
+        <v>0.79574509803921578</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30" s="11">
+        <f t="shared" si="1"/>
+        <v>0.21666666666666667</v>
+      </c>
+      <c r="C30" s="11">
+        <f t="shared" si="1"/>
+        <v>0.14799999999999999</v>
+      </c>
+      <c r="D30" s="11">
+        <f t="shared" si="1"/>
+        <v>8.2500000000000004E-2</v>
+      </c>
+      <c r="E30" s="11">
+        <f t="shared" si="2"/>
+        <v>3.793103448275862E-2</v>
+      </c>
+      <c r="F30" s="11">
+        <f t="shared" si="1"/>
+        <v>0.2513333333333333</v>
+      </c>
+      <c r="G30" s="10">
+        <f t="shared" si="3"/>
+        <v>0.73643103448275871</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63C902CE-5066-45BF-BEA2-646F8D396124}">
+  <dimension ref="A1:G26"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="21" customWidth="1"/>
+    <col min="2" max="2" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A1" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F1" s="6" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2">
+        <v>340</v>
+      </c>
+      <c r="C2">
+        <v>33</v>
+      </c>
+      <c r="D2">
+        <f>IF('Średnie autobusy'!D3="",0, LEN('Średnie autobusy'!D3) - LEN(SUBSTITUTE('Średnie autobusy'!D3,",",""))+1)</f>
+        <v>3</v>
+      </c>
+      <c r="E2">
+        <v>2.6</v>
+      </c>
+      <c r="F2" s="7">
+        <f>AVERAGE(6,4,2)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3">
+        <v>218</v>
+      </c>
+      <c r="C3">
+        <v>27</v>
+      </c>
+      <c r="D3">
+        <f>IF('Średnie autobusy'!D4="",0, LEN('Średnie autobusy'!D4) - LEN(SUBSTITUTE('Średnie autobusy'!D4,",",""))+1)</f>
+        <v>4</v>
+      </c>
+      <c r="E3">
+        <v>2.4</v>
+      </c>
+      <c r="F3" s="7">
+        <f>AVERAGE(6,8,10)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4">
+        <v>250</v>
+      </c>
+      <c r="C4">
+        <v>33</v>
+      </c>
+      <c r="D4">
+        <f>IF('Średnie autobusy'!D5="",0, LEN('Średnie autobusy'!D5) - LEN(SUBSTITUTE('Średnie autobusy'!D5,",",""))+1)</f>
+        <v>4</v>
+      </c>
+      <c r="E4">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="F4" s="7">
+        <f>AVERAGE(10,5,5)</f>
+        <v>6.666666666666667</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5">
+        <v>326</v>
+      </c>
+      <c r="C5">
+        <v>36</v>
+      </c>
+      <c r="D5">
+        <f>IF('Średnie autobusy'!D7="",0, LEN('Średnie autobusy'!D7) - LEN(SUBSTITUTE('Średnie autobusy'!D7,",",""))+1)</f>
+        <v>4</v>
+      </c>
+      <c r="E5">
+        <v>2.6</v>
+      </c>
+      <c r="F5" s="7">
+        <f>AVERAGE(5,5,5)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>19</v>
+      </c>
+      <c r="B6">
+        <v>210</v>
+      </c>
+      <c r="C6">
+        <v>16</v>
+      </c>
+      <c r="D6">
+        <f>IF('Średnie autobusy'!D9="",0, LEN('Średnie autobusy'!D9) - LEN(SUBSTITUTE('Średnie autobusy'!D9,",",""))+1)</f>
+        <v>4</v>
+      </c>
+      <c r="E6">
+        <v>0.6</v>
+      </c>
+      <c r="F6" s="7">
+        <f>AVERAGE(3,6,4)</f>
+        <v>4.333333333333333</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7">
+        <v>340</v>
+      </c>
+      <c r="C7">
+        <v>24</v>
+      </c>
+      <c r="D7">
+        <f>IF('Średnie autobusy'!D10="",0, LEN('Średnie autobusy'!D10) - LEN(SUBSTITUTE('Średnie autobusy'!D10,",",""))+1)</f>
+        <v>4</v>
+      </c>
+      <c r="E7">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="F7" s="7">
+        <f>AVERAGE(5,6,4)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8">
+        <v>247</v>
+      </c>
+      <c r="C8">
+        <v>26</v>
+      </c>
+      <c r="D8">
+        <f>IF('Średnie autobusy'!D11="",0, LEN('Średnie autobusy'!D11) - LEN(SUBSTITUTE('Średnie autobusy'!D11,",",""))+1)</f>
+        <v>3</v>
+      </c>
+      <c r="E8">
+        <v>0.9</v>
+      </c>
+      <c r="F8" s="7">
+        <f>AVERAGE(5,7,5)</f>
+        <v>5.666666666666667</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B9">
+        <v>299</v>
+      </c>
+      <c r="C9">
+        <v>32</v>
+      </c>
+      <c r="D9">
+        <f>IF('Średnie autobusy'!D13="",0, LEN('Średnie autobusy'!D13) - LEN(SUBSTITUTE('Średnie autobusy'!D13,",",""))+1)</f>
+        <v>5</v>
+      </c>
+      <c r="E9">
+        <v>1.3</v>
+      </c>
+      <c r="F9" s="7">
+        <f>AVERAGE(9,9,7)</f>
+        <v>8.3333333333333339</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>33</v>
+      </c>
+      <c r="B10">
+        <v>330</v>
+      </c>
+      <c r="C10">
+        <v>29</v>
+      </c>
+      <c r="D10">
+        <f>IF('Średnie autobusy'!D15="",0, LEN('Średnie autobusy'!D15) - LEN(SUBSTITUTE('Średnie autobusy'!D15,",",""))+1)</f>
+        <v>4</v>
+      </c>
+      <c r="E10">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="F10" s="7">
+        <f>AVERAGE(9,7,10)</f>
+        <v>8.6666666666666661</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11">
+        <v>360</v>
+      </c>
+      <c r="C11">
+        <v>47</v>
+      </c>
+      <c r="D11">
+        <f>IF('Średnie autobusy'!D16="",0, LEN('Średnie autobusy'!D16) - LEN(SUBSTITUTE('Średnie autobusy'!D16,",",""))+1)</f>
+        <v>3</v>
+      </c>
+      <c r="E11">
+        <v>0.9</v>
+      </c>
+      <c r="F11" s="7">
+        <f>AVERAGE(8,3,8)</f>
+        <v>6.333333333333333</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>46</v>
+      </c>
+      <c r="B13">
+        <f>MAX(B2:B11)</f>
+        <v>360</v>
+      </c>
+      <c r="C13">
+        <f>MAX(C2:C11)</f>
+        <v>47</v>
+      </c>
+      <c r="D13">
+        <f>MAX(D2:D11)</f>
+        <v>5</v>
+      </c>
+      <c r="E13">
+        <f>MIN(E2:E11)</f>
+        <v>0.6</v>
+      </c>
+      <c r="F13" s="7">
+        <f>MAX(F2:F11)</f>
+        <v>8.6666666666666661</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14">
+        <v>0.26</v>
+      </c>
+      <c r="C14">
+        <v>0.26</v>
+      </c>
+      <c r="D14">
+        <v>0.11</v>
+      </c>
+      <c r="E14">
+        <v>0.11</v>
+      </c>
+      <c r="F14">
+        <v>0.26</v>
+      </c>
+      <c r="G14">
+        <f>SUM(B14:F14)</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A16" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>15</v>
+      </c>
+      <c r="B17" s="11">
+        <f>(B2/B$13)*B$14</f>
+        <v>0.24555555555555555</v>
+      </c>
+      <c r="C17" s="11">
+        <f t="shared" ref="C17:F17" si="0">(C2/C$13)*C$14</f>
+        <v>0.18255319148936172</v>
+      </c>
+      <c r="D17" s="11">
+        <f t="shared" si="0"/>
+        <v>6.6000000000000003E-2</v>
+      </c>
+      <c r="E17" s="11">
+        <f>($E$13/E2)*$E$14</f>
+        <v>2.5384615384615384E-2</v>
+      </c>
+      <c r="F17" s="11">
+        <f t="shared" si="0"/>
+        <v>0.12000000000000001</v>
+      </c>
+      <c r="G17" s="10">
+        <f>SUM(B17:F17)</f>
+        <v>0.6394933624295327</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="11">
+        <f t="shared" ref="B18:F26" si="1">(B3/B$13)*B$14</f>
+        <v>0.15744444444444444</v>
+      </c>
+      <c r="C18" s="11">
+        <f t="shared" si="1"/>
+        <v>0.14936170212765959</v>
+      </c>
+      <c r="D18" s="11">
+        <f t="shared" si="1"/>
+        <v>8.8000000000000009E-2</v>
+      </c>
+      <c r="E18" s="11">
+        <f t="shared" ref="E18:E26" si="2">($E$13/E3)*$E$14</f>
+        <v>2.75E-2</v>
+      </c>
+      <c r="F18" s="11">
+        <f t="shared" si="1"/>
+        <v>0.24000000000000002</v>
+      </c>
+      <c r="G18" s="10">
+        <f t="shared" ref="G18:G26" si="3">SUM(B18:F18)</f>
+        <v>0.66230614657210407</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="11">
+        <f t="shared" si="1"/>
+        <v>0.18055555555555555</v>
+      </c>
+      <c r="C19" s="11">
+        <f t="shared" si="1"/>
+        <v>0.18255319148936172</v>
+      </c>
+      <c r="D19" s="11">
+        <f t="shared" si="1"/>
+        <v>8.8000000000000009E-2</v>
+      </c>
+      <c r="E19" s="11">
+        <f t="shared" si="2"/>
+        <v>0.06</v>
+      </c>
+      <c r="F19" s="11">
+        <f t="shared" si="1"/>
+        <v>0.2</v>
+      </c>
+      <c r="G19" s="10">
+        <f t="shared" si="3"/>
+        <v>0.71110874704491733</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" s="11">
+        <f t="shared" si="1"/>
+        <v>0.23544444444444446</v>
+      </c>
+      <c r="C20" s="11">
+        <f t="shared" si="1"/>
+        <v>0.19914893617021276</v>
+      </c>
+      <c r="D20" s="11">
+        <f t="shared" si="1"/>
+        <v>8.8000000000000009E-2</v>
+      </c>
+      <c r="E20" s="11">
+        <f t="shared" si="2"/>
+        <v>2.5384615384615384E-2</v>
+      </c>
+      <c r="F20" s="11">
+        <f t="shared" si="1"/>
+        <v>0.15000000000000002</v>
+      </c>
+      <c r="G20" s="10">
+        <f t="shared" si="3"/>
+        <v>0.69797799599927257</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="11">
+        <f t="shared" si="1"/>
+        <v>0.15166666666666667</v>
+      </c>
+      <c r="C21" s="11">
+        <f t="shared" si="1"/>
+        <v>8.851063829787234E-2</v>
+      </c>
+      <c r="D21" s="11">
+        <f t="shared" si="1"/>
+        <v>8.8000000000000009E-2</v>
+      </c>
+      <c r="E21" s="11">
+        <f t="shared" si="2"/>
+        <v>0.11</v>
+      </c>
+      <c r="F21" s="11">
+        <f t="shared" si="1"/>
+        <v>0.13</v>
+      </c>
+      <c r="G21" s="10">
+        <f t="shared" si="3"/>
+        <v>0.568177304964539</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="11">
+        <f t="shared" si="1"/>
+        <v>0.24555555555555555</v>
+      </c>
+      <c r="C22" s="11">
+        <f t="shared" si="1"/>
+        <v>0.1327659574468085</v>
+      </c>
+      <c r="D22" s="11">
+        <f t="shared" si="1"/>
+        <v>8.8000000000000009E-2</v>
+      </c>
+      <c r="E22" s="11">
+        <f t="shared" si="2"/>
+        <v>0.03</v>
+      </c>
+      <c r="F22" s="11">
+        <f t="shared" si="1"/>
+        <v>0.15000000000000002</v>
+      </c>
+      <c r="G22" s="10">
+        <f t="shared" si="3"/>
+        <v>0.64632151300236407</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A23" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="11">
+        <f t="shared" si="1"/>
+        <v>0.1783888888888889</v>
+      </c>
+      <c r="C23" s="11">
+        <f t="shared" si="1"/>
+        <v>0.14382978723404255</v>
+      </c>
+      <c r="D23" s="11">
+        <f t="shared" si="1"/>
+        <v>6.6000000000000003E-2</v>
+      </c>
+      <c r="E23" s="11">
+        <f t="shared" si="2"/>
+        <v>7.3333333333333334E-2</v>
+      </c>
+      <c r="F23" s="11">
+        <f t="shared" si="1"/>
+        <v>0.17000000000000004</v>
+      </c>
+      <c r="G23" s="10">
+        <f t="shared" si="3"/>
+        <v>0.63155200945626477</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" s="11">
+        <f t="shared" si="1"/>
+        <v>0.21594444444444447</v>
+      </c>
+      <c r="C24" s="11">
+        <f t="shared" si="1"/>
+        <v>0.17702127659574468</v>
+      </c>
+      <c r="D24" s="11">
+        <f t="shared" si="1"/>
+        <v>0.11</v>
+      </c>
+      <c r="E24" s="11">
+        <f t="shared" si="2"/>
+        <v>5.0769230769230768E-2</v>
+      </c>
+      <c r="F24" s="11">
+        <f t="shared" si="1"/>
+        <v>0.25000000000000006</v>
+      </c>
+      <c r="G24" s="10">
+        <f t="shared" si="3"/>
+        <v>0.8037349518094199</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" s="11">
+        <f t="shared" si="1"/>
+        <v>0.23833333333333334</v>
+      </c>
+      <c r="C25" s="11">
+        <f t="shared" si="1"/>
+        <v>0.16042553191489362</v>
+      </c>
+      <c r="D25" s="11">
+        <f t="shared" si="1"/>
+        <v>8.8000000000000009E-2</v>
+      </c>
+      <c r="E25" s="11">
+        <f t="shared" si="2"/>
+        <v>0.06</v>
+      </c>
+      <c r="F25" s="11">
+        <f t="shared" si="1"/>
+        <v>0.26</v>
+      </c>
+      <c r="G25" s="10">
+        <f t="shared" si="3"/>
+        <v>0.80675886524822693</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A26" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="B26" s="14">
+        <f t="shared" si="1"/>
+        <v>0.26</v>
+      </c>
+      <c r="C26" s="14">
+        <f t="shared" si="1"/>
+        <v>0.26</v>
+      </c>
+      <c r="D26" s="14">
+        <f t="shared" si="1"/>
+        <v>6.6000000000000003E-2</v>
+      </c>
+      <c r="E26" s="14">
+        <f t="shared" si="2"/>
+        <v>7.3333333333333334E-2</v>
+      </c>
+      <c r="F26" s="14">
+        <f t="shared" si="1"/>
+        <v>0.19000000000000003</v>
+      </c>
+      <c r="G26" s="12">
+        <f t="shared" si="3"/>
+        <v>0.8493333333333335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
dane autobusów + analiza SAW + tabele przestawne
</commit_message>
<xml_diff>
--- a/autobusy.xlsx
+++ b/autobusy.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\teste\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7B6CF2B-388F-4410-B130-D259FB8112F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4AECBBC-3EB4-412C-AC16-8DC4DD893F88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{78F6C6CF-C9FD-4C30-A6D3-8F4A203AF3AD}"/>
   </bookViews>
@@ -19,6 +19,10 @@
     <sheet name="Średnie autobusy (2)" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <pivotCaches>
+    <pivotCache cacheId="3" r:id="rId5"/>
+    <pivotCache cacheId="7" r:id="rId6"/>
+  </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -42,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="57">
   <si>
     <t>Model</t>
   </si>
@@ -192,6 +196,27 @@
   </si>
   <si>
     <t>Waga</t>
+  </si>
+  <si>
+    <t>moc silnika</t>
+  </si>
+  <si>
+    <t>miejsca pasażerów</t>
+  </si>
+  <si>
+    <t>udogodnienia niepełnosprawnych</t>
+  </si>
+  <si>
+    <t>koszty zakupu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prestiż </t>
+  </si>
+  <si>
+    <t>wartość SAW</t>
+  </si>
+  <si>
+    <t>model</t>
   </si>
 </sst>
 </file>
@@ -200,7 +225,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="8" formatCode="#,##0.00\ &quot;zł&quot;;[Red]\-#,##0.00\ &quot;zł&quot;"/>
-    <numFmt numFmtId="167" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -258,7 +283,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -268,12 +293,15 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -289,6 +317,544 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Patryk Klimek" refreshedDate="46183.497629398145" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="10" xr:uid="{FC30D319-B356-4460-A3AB-822B9CA51265}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A16:G26" sheet="Średnie autobusy (2)"/>
+  </cacheSource>
+  <cacheFields count="7">
+    <cacheField name="Model" numFmtId="0">
+      <sharedItems count="10">
+        <s v="Urbino 10,5 electric"/>
+        <s v="Urbino 8,9 LE electric"/>
+        <s v="Urbino 8,9 LE"/>
+        <s v="MAN Lion's City 10 E"/>
+        <s v="SANCITY 9LE"/>
+        <s v="SANCITY 10LFE"/>
+        <s v="SANCITY 10LF"/>
+        <s v="Citaro K"/>
+        <s v="Crossway 10.8LE"/>
+        <s v="Crossway Pro 10,8"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="moc silnika [KM]" numFmtId="2">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.15166666666666667" maxValue="0.26"/>
+    </cacheField>
+    <cacheField name="miejsca dla pasażerów" numFmtId="2">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="8.851063829787234E-2" maxValue="0.26"/>
+    </cacheField>
+    <cacheField name="udogodnienia dla niepełnosprawnych" numFmtId="2">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="6.6000000000000003E-2" maxValue="0.11"/>
+    </cacheField>
+    <cacheField name="koszt zakupu" numFmtId="2">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="2.5384615384615384E-2" maxValue="0.11"/>
+    </cacheField>
+    <cacheField name="prestiż" numFmtId="2">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.12000000000000001" maxValue="0.26"/>
+    </cacheField>
+    <cacheField name="SAW" numFmtId="164">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.568177304964539" maxValue="0.8493333333333335"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Patryk Klimek" refreshedDate="46183.50246909722" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="12" xr:uid="{532C073B-53B9-43CD-B7E0-817ECB39F861}">
+  <cacheSource type="worksheet">
+    <worksheetSource ref="A18:G30" sheet="Duże autobusy (2)"/>
+  </cacheSource>
+  <cacheFields count="7">
+    <cacheField name="Model" numFmtId="0">
+      <sharedItems count="12">
+        <s v="Urbino 15 LE electric"/>
+        <s v="Urbino 18 CNG"/>
+        <s v="Urbino 18"/>
+        <s v="Urbino 12"/>
+        <s v="Urbino 12 CNG"/>
+        <s v="MAN Lion's City 12 E"/>
+        <s v="MAN Lion's Intercity LE 14"/>
+        <s v="MAN Lion's City 12 G"/>
+        <s v="SANCITY 12LFH"/>
+        <s v="SANCITY 12LF"/>
+        <s v="CapaCity L"/>
+        <s v="Nesobus 12"/>
+      </sharedItems>
+    </cacheField>
+    <cacheField name="moc silnika [KM]" numFmtId="2">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.16313725490196079" maxValue="0.26"/>
+    </cacheField>
+    <cacheField name="miejsca dla pasażerów" numFmtId="2">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="6.4000000000000001E-2" maxValue="0.26"/>
+    </cacheField>
+    <cacheField name="udogodnienia dla niepełnosprawnych" numFmtId="2">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="5.5E-2" maxValue="0.11"/>
+    </cacheField>
+    <cacheField name="koszt zakupu" numFmtId="2">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="3.3846153846153845E-2" maxValue="0.11"/>
+    </cacheField>
+    <cacheField name="prestiż" numFmtId="2">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="7.8E-2" maxValue="0.26"/>
+    </cacheField>
+    <cacheField name="SAW" numFmtId="164">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" minValue="0.56943137254901954" maxValue="0.81225490196078431"/>
+    </cacheField>
+  </cacheFields>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
+      <x14:pivotCacheDefinition/>
+    </ext>
+  </extLst>
+</pivotCacheDefinition>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="10">
+  <r>
+    <x v="0"/>
+    <n v="0.24555555555555555"/>
+    <n v="0.18255319148936172"/>
+    <n v="6.6000000000000003E-2"/>
+    <n v="2.5384615384615384E-2"/>
+    <n v="0.12000000000000001"/>
+    <n v="0.6394933624295327"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <n v="0.15744444444444444"/>
+    <n v="0.14936170212765959"/>
+    <n v="8.8000000000000009E-2"/>
+    <n v="2.75E-2"/>
+    <n v="0.24000000000000002"/>
+    <n v="0.66230614657210407"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <n v="0.18055555555555555"/>
+    <n v="0.18255319148936172"/>
+    <n v="8.8000000000000009E-2"/>
+    <n v="0.06"/>
+    <n v="0.2"/>
+    <n v="0.71110874704491733"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <n v="0.23544444444444446"/>
+    <n v="0.19914893617021276"/>
+    <n v="8.8000000000000009E-2"/>
+    <n v="2.5384615384615384E-2"/>
+    <n v="0.15000000000000002"/>
+    <n v="0.69797799599927257"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <n v="0.15166666666666667"/>
+    <n v="8.851063829787234E-2"/>
+    <n v="8.8000000000000009E-2"/>
+    <n v="0.11"/>
+    <n v="0.13"/>
+    <n v="0.568177304964539"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <n v="0.24555555555555555"/>
+    <n v="0.1327659574468085"/>
+    <n v="8.8000000000000009E-2"/>
+    <n v="0.03"/>
+    <n v="0.15000000000000002"/>
+    <n v="0.64632151300236407"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <n v="0.1783888888888889"/>
+    <n v="0.14382978723404255"/>
+    <n v="6.6000000000000003E-2"/>
+    <n v="7.3333333333333334E-2"/>
+    <n v="0.17000000000000004"/>
+    <n v="0.63155200945626477"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <n v="0.21594444444444447"/>
+    <n v="0.17702127659574468"/>
+    <n v="0.11"/>
+    <n v="5.0769230769230768E-2"/>
+    <n v="0.25000000000000006"/>
+    <n v="0.8037349518094199"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <n v="0.23833333333333334"/>
+    <n v="0.16042553191489362"/>
+    <n v="8.8000000000000009E-2"/>
+    <n v="0.06"/>
+    <n v="0.26"/>
+    <n v="0.80675886524822693"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <n v="0.26"/>
+    <n v="0.26"/>
+    <n v="6.6000000000000003E-2"/>
+    <n v="7.3333333333333334E-2"/>
+    <n v="0.19000000000000003"/>
+    <n v="0.8493333333333335"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotCache/pivotCacheRecords2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="12">
+  <r>
+    <x v="0"/>
+    <n v="0.26"/>
+    <n v="0.26"/>
+    <n v="5.5E-2"/>
+    <n v="4.9999999999999996E-2"/>
+    <n v="0.182"/>
+    <n v="0.80700000000000016"/>
+  </r>
+  <r>
+    <x v="1"/>
+    <n v="0.20392156862745098"/>
+    <n v="0.22"/>
+    <n v="8.2500000000000004E-2"/>
+    <n v="4.5833333333333337E-2"/>
+    <n v="0.26"/>
+    <n v="0.81225490196078431"/>
+  </r>
+  <r>
+    <x v="2"/>
+    <n v="0.19754901960784313"/>
+    <n v="0.21600000000000003"/>
+    <n v="8.2500000000000004E-2"/>
+    <n v="6.1111111111111116E-2"/>
+    <n v="0.16466666666666666"/>
+    <n v="0.72182679738562094"/>
+  </r>
+  <r>
+    <x v="3"/>
+    <n v="0.16313725490196079"/>
+    <n v="6.4000000000000001E-2"/>
+    <n v="8.2500000000000004E-2"/>
+    <n v="0.11"/>
+    <n v="0.22533333333333333"/>
+    <n v="0.64497058823529407"/>
+  </r>
+  <r>
+    <x v="4"/>
+    <n v="0.20392156862745098"/>
+    <n v="0.16"/>
+    <n v="8.2500000000000004E-2"/>
+    <n v="9.9999999999999992E-2"/>
+    <n v="0.12133333333333333"/>
+    <n v="0.66775490196078424"/>
+  </r>
+  <r>
+    <x v="5"/>
+    <n v="0.2077450980392157"/>
+    <n v="0.17600000000000002"/>
+    <n v="0.11"/>
+    <n v="4.2307692307692303E-2"/>
+    <n v="0.16466666666666666"/>
+    <n v="0.70071945701357463"/>
+  </r>
+  <r>
+    <x v="6"/>
+    <n v="0.16887254901960785"/>
+    <n v="0.252"/>
+    <n v="8.2500000000000004E-2"/>
+    <n v="6.1111111111111116E-2"/>
+    <n v="0.16466666666666666"/>
+    <n v="0.72915032679738556"/>
+  </r>
+  <r>
+    <x v="7"/>
+    <n v="0.17843137254901961"/>
+    <n v="0.14799999999999999"/>
+    <n v="0.11"/>
+    <n v="5.5E-2"/>
+    <n v="7.8E-2"/>
+    <n v="0.56943137254901954"/>
+  </r>
+  <r>
+    <x v="8"/>
+    <n v="0.21921568627450982"/>
+    <n v="0.16"/>
+    <n v="8.2500000000000004E-2"/>
+    <n v="3.3846153846153845E-2"/>
+    <n v="0.20800000000000002"/>
+    <n v="0.70356184012066381"/>
+  </r>
+  <r>
+    <x v="9"/>
+    <n v="0.17651960784313728"/>
+    <n v="0.16"/>
+    <n v="8.2500000000000004E-2"/>
+    <n v="0.11"/>
+    <n v="0.10400000000000001"/>
+    <n v="0.63301960784313727"/>
+  </r>
+  <r>
+    <x v="10"/>
+    <n v="0.22941176470588234"/>
+    <n v="0.17600000000000002"/>
+    <n v="0.11"/>
+    <n v="5.5E-2"/>
+    <n v="0.22533333333333333"/>
+    <n v="0.79574509803921578"/>
+  </r>
+  <r>
+    <x v="11"/>
+    <n v="0.21666666666666667"/>
+    <n v="0.14799999999999999"/>
+    <n v="8.2500000000000004E-2"/>
+    <n v="3.793103448275862E-2"/>
+    <n v="0.2513333333333333"/>
+    <n v="0.73643103448275871"/>
+  </r>
+</pivotCacheRecords>
+</file>
+
+<file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{07181233-C502-43AB-8A2B-E089A1637B81}" name="Tabela przestawna2" cacheId="7" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Wartości" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="Model">
+  <location ref="A33:G45" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="7">
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="13">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="11"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="5"/>
+        <item x="10"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="5"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField dataField="1" numFmtId="2" showAll="0"/>
+    <pivotField dataField="1" numFmtId="2" showAll="0"/>
+    <pivotField dataField="1" numFmtId="2" showAll="0"/>
+    <pivotField dataField="1" numFmtId="2" showAll="0"/>
+    <pivotField dataField="1" numFmtId="2" showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="12">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="11"/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="10"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+    <i i="3">
+      <x v="3"/>
+    </i>
+    <i i="4">
+      <x v="4"/>
+    </i>
+    <i i="5">
+      <x v="5"/>
+    </i>
+  </colItems>
+  <dataFields count="6">
+    <dataField name="moc silnika" fld="1" baseField="0" baseItem="0" numFmtId="2"/>
+    <dataField name="miejsca pasażerów" fld="2" baseField="0" baseItem="0" numFmtId="2"/>
+    <dataField name="udogodnienia niepełnosprawnych" fld="3" baseField="0" baseItem="0" numFmtId="2"/>
+    <dataField name="koszty zakupu" fld="4" baseField="0" baseItem="0" numFmtId="2"/>
+    <dataField name="prestiż " fld="5" baseField="0" baseItem="0" numFmtId="2"/>
+    <dataField name="wartość SAW" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{7CB3FD6C-AFC4-4B07-B04C-578360CBD737}" name="Tabela przestawna1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Wartości" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" rowHeaderCaption="model">
+  <location ref="A29:G39" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="7">
+    <pivotField axis="axisRow" showAll="0" sortType="descending">
+      <items count="11">
+        <item x="1"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="3"/>
+        <item x="9"/>
+        <item x="8"/>
+        <item x="7"/>
+        <item t="default"/>
+      </items>
+      <autoSortScope>
+        <pivotArea dataOnly="0" outline="0" fieldPosition="0">
+          <references count="1">
+            <reference field="4294967294" count="1" selected="0">
+              <x v="5"/>
+            </reference>
+          </references>
+        </pivotArea>
+      </autoSortScope>
+    </pivotField>
+    <pivotField dataField="1" numFmtId="2" showAll="0"/>
+    <pivotField dataField="1" numFmtId="2" showAll="0"/>
+    <pivotField dataField="1" numFmtId="2" showAll="0"/>
+    <pivotField dataField="1" numFmtId="2" showAll="0"/>
+    <pivotField dataField="1" numFmtId="2" showAll="0"/>
+    <pivotField dataField="1" numFmtId="164" showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="0"/>
+  </rowFields>
+  <rowItems count="10">
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="8"/>
+    </i>
+    <i>
+      <x v="9"/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="6"/>
+    </i>
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="5"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+  </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+    <i i="2">
+      <x v="2"/>
+    </i>
+    <i i="3">
+      <x v="3"/>
+    </i>
+    <i i="4">
+      <x v="4"/>
+    </i>
+    <i i="5">
+      <x v="5"/>
+    </i>
+  </colItems>
+  <dataFields count="6">
+    <dataField name="moc silnika" fld="1" baseField="0" baseItem="0" numFmtId="2"/>
+    <dataField name="miejsca pasażerów" fld="2" baseField="0" baseItem="0" numFmtId="2"/>
+    <dataField name="udogodnienia niepełnosprawnych" fld="3" baseField="0" baseItem="0" numFmtId="2"/>
+    <dataField name="koszty zakupu" fld="4" baseField="0" baseItem="0" numFmtId="2"/>
+    <dataField name="prestiż " fld="5" baseField="0" baseItem="0" numFmtId="2"/>
+    <dataField name="wartość SAW" fld="6" baseField="0" baseItem="0" numFmtId="164"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1135,7 +1701,7 @@
       <c r="C10">
         <v>24</v>
       </c>
-      <c r="D10" s="9" t="s">
+      <c r="D10" t="s">
         <v>36</v>
       </c>
       <c r="E10">
@@ -1239,7 +1805,7 @@
       <c r="C16">
         <v>47</v>
       </c>
-      <c r="D16" s="9" t="s">
+      <c r="D16" t="s">
         <v>40</v>
       </c>
       <c r="E16">
@@ -1257,16 +1823,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF33C538-C2CB-4E1F-B5CA-2C4D84AF0445}">
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I45"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="23.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.453125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.81640625" customWidth="1"/>
-    <col min="5" max="5" width="23.36328125" customWidth="1"/>
-    <col min="6" max="6" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.26953125" customWidth="1"/>
+    <col min="1" max="1" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="39.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.81640625" customWidth="1"/>
     <col min="9" max="9" width="10.81640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1632,56 +2198,56 @@
       <c r="A19" t="s">
         <v>4</v>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="10">
         <f>(B2/B$15)*B$16</f>
         <v>0.26</v>
       </c>
-      <c r="C19" s="11">
+      <c r="C19" s="10">
         <f t="shared" ref="C19:F19" si="0">(C2/C$15)*C$16</f>
         <v>0.26</v>
       </c>
-      <c r="D19" s="11">
+      <c r="D19" s="10">
         <f t="shared" si="0"/>
         <v>5.5E-2</v>
       </c>
-      <c r="E19" s="11">
+      <c r="E19" s="10">
         <f>($E$15/E2)*$E$16</f>
         <v>4.9999999999999996E-2</v>
       </c>
-      <c r="F19" s="11">
+      <c r="F19" s="10">
         <f t="shared" si="0"/>
         <v>0.182</v>
       </c>
-      <c r="G19" s="10">
+      <c r="G19" s="9">
         <f>SUM(B19:F19)</f>
         <v>0.80700000000000016</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="B20" s="14">
+      <c r="B20" s="13">
         <f t="shared" ref="B20:F30" si="1">(B3/B$15)*B$16</f>
         <v>0.20392156862745098</v>
       </c>
-      <c r="C20" s="14">
+      <c r="C20" s="13">
         <f t="shared" si="1"/>
         <v>0.22</v>
       </c>
-      <c r="D20" s="14">
+      <c r="D20" s="13">
         <f t="shared" si="1"/>
         <v>8.2500000000000004E-2</v>
       </c>
-      <c r="E20" s="14">
+      <c r="E20" s="13">
         <f t="shared" ref="E20:E30" si="2">($E$15/E3)*$E$16</f>
         <v>4.5833333333333337E-2</v>
       </c>
-      <c r="F20" s="14">
+      <c r="F20" s="13">
         <f t="shared" si="1"/>
         <v>0.26</v>
       </c>
-      <c r="G20" s="12">
+      <c r="G20" s="11">
         <f t="shared" ref="G20:G30" si="3">SUM(B20:F20)</f>
         <v>0.81225490196078431</v>
       </c>
@@ -1690,27 +2256,27 @@
       <c r="A21" t="s">
         <v>6</v>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="10">
         <f t="shared" si="1"/>
         <v>0.19754901960784313</v>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="10">
         <f t="shared" si="1"/>
         <v>0.21600000000000003</v>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="10">
         <f t="shared" si="1"/>
         <v>8.2500000000000004E-2</v>
       </c>
-      <c r="E21" s="11">
+      <c r="E21" s="10">
         <f t="shared" si="2"/>
         <v>6.1111111111111116E-2</v>
       </c>
-      <c r="F21" s="11">
+      <c r="F21" s="10">
         <f t="shared" si="1"/>
         <v>0.16466666666666666</v>
       </c>
-      <c r="G21" s="10">
+      <c r="G21" s="9">
         <f t="shared" si="3"/>
         <v>0.72182679738562094</v>
       </c>
@@ -1719,27 +2285,27 @@
       <c r="A22" t="s">
         <v>7</v>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="10">
         <f t="shared" si="1"/>
         <v>0.16313725490196079</v>
       </c>
-      <c r="C22" s="11">
+      <c r="C22" s="10">
         <f t="shared" si="1"/>
         <v>6.4000000000000001E-2</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="10">
         <f t="shared" si="1"/>
         <v>8.2500000000000004E-2</v>
       </c>
-      <c r="E22" s="11">
+      <c r="E22" s="10">
         <f t="shared" si="2"/>
         <v>0.11</v>
       </c>
-      <c r="F22" s="11">
+      <c r="F22" s="10">
         <f t="shared" si="1"/>
         <v>0.22533333333333333</v>
       </c>
-      <c r="G22" s="10">
+      <c r="G22" s="9">
         <f t="shared" si="3"/>
         <v>0.64497058823529407</v>
       </c>
@@ -1748,27 +2314,27 @@
       <c r="A23" t="s">
         <v>8</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="10">
         <f t="shared" si="1"/>
         <v>0.20392156862745098</v>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="10">
         <f t="shared" si="1"/>
         <v>0.16</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="10">
         <f t="shared" si="1"/>
         <v>8.2500000000000004E-2</v>
       </c>
-      <c r="E23" s="11">
+      <c r="E23" s="10">
         <f t="shared" si="2"/>
         <v>9.9999999999999992E-2</v>
       </c>
-      <c r="F23" s="11">
+      <c r="F23" s="10">
         <f t="shared" si="1"/>
         <v>0.12133333333333333</v>
       </c>
-      <c r="G23" s="10">
+      <c r="G23" s="9">
         <f t="shared" si="3"/>
         <v>0.66775490196078424</v>
       </c>
@@ -1777,27 +2343,27 @@
       <c r="A24" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="10">
         <f t="shared" si="1"/>
         <v>0.2077450980392157</v>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="10">
         <f t="shared" si="1"/>
         <v>0.17600000000000002</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="10">
         <f t="shared" si="1"/>
         <v>0.11</v>
       </c>
-      <c r="E24" s="11">
+      <c r="E24" s="10">
         <f t="shared" si="2"/>
         <v>4.2307692307692303E-2</v>
       </c>
-      <c r="F24" s="11">
+      <c r="F24" s="10">
         <f t="shared" si="1"/>
         <v>0.16466666666666666</v>
       </c>
-      <c r="G24" s="10">
+      <c r="G24" s="9">
         <f t="shared" si="3"/>
         <v>0.70071945701357463</v>
       </c>
@@ -1806,27 +2372,27 @@
       <c r="A25" t="s">
         <v>27</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="10">
         <f t="shared" si="1"/>
         <v>0.16887254901960785</v>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="10">
         <f t="shared" si="1"/>
         <v>0.252</v>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="10">
         <f t="shared" si="1"/>
         <v>8.2500000000000004E-2</v>
       </c>
-      <c r="E25" s="11">
+      <c r="E25" s="10">
         <f t="shared" si="2"/>
         <v>6.1111111111111116E-2</v>
       </c>
-      <c r="F25" s="11">
+      <c r="F25" s="10">
         <f t="shared" si="1"/>
         <v>0.16466666666666666</v>
       </c>
-      <c r="G25" s="10">
+      <c r="G25" s="9">
         <f t="shared" si="3"/>
         <v>0.72915032679738556</v>
       </c>
@@ -1835,27 +2401,27 @@
       <c r="A26" t="s">
         <v>28</v>
       </c>
-      <c r="B26" s="11">
+      <c r="B26" s="10">
         <f t="shared" si="1"/>
         <v>0.17843137254901961</v>
       </c>
-      <c r="C26" s="11">
+      <c r="C26" s="10">
         <f t="shared" si="1"/>
         <v>0.14799999999999999</v>
       </c>
-      <c r="D26" s="11">
+      <c r="D26" s="10">
         <f t="shared" si="1"/>
         <v>0.11</v>
       </c>
-      <c r="E26" s="11">
+      <c r="E26" s="10">
         <f t="shared" si="2"/>
         <v>5.5E-2</v>
       </c>
-      <c r="F26" s="11">
+      <c r="F26" s="10">
         <f t="shared" si="1"/>
         <v>7.8E-2</v>
       </c>
-      <c r="G26" s="10">
+      <c r="G26" s="9">
         <f t="shared" si="3"/>
         <v>0.56943137254901954</v>
       </c>
@@ -1864,27 +2430,27 @@
       <c r="A27" t="s">
         <v>11</v>
       </c>
-      <c r="B27" s="11">
+      <c r="B27" s="10">
         <f t="shared" si="1"/>
         <v>0.21921568627450982</v>
       </c>
-      <c r="C27" s="11">
+      <c r="C27" s="10">
         <f t="shared" si="1"/>
         <v>0.16</v>
       </c>
-      <c r="D27" s="11">
+      <c r="D27" s="10">
         <f t="shared" si="1"/>
         <v>8.2500000000000004E-2</v>
       </c>
-      <c r="E27" s="11">
+      <c r="E27" s="10">
         <f t="shared" si="2"/>
         <v>3.3846153846153845E-2</v>
       </c>
-      <c r="F27" s="11">
+      <c r="F27" s="10">
         <f t="shared" si="1"/>
         <v>0.20800000000000002</v>
       </c>
-      <c r="G27" s="10">
+      <c r="G27" s="9">
         <f t="shared" si="3"/>
         <v>0.70356184012066381</v>
       </c>
@@ -1893,27 +2459,27 @@
       <c r="A28" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="11">
+      <c r="B28" s="10">
         <f t="shared" si="1"/>
         <v>0.17651960784313728</v>
       </c>
-      <c r="C28" s="11">
+      <c r="C28" s="10">
         <f t="shared" si="1"/>
         <v>0.16</v>
       </c>
-      <c r="D28" s="11">
+      <c r="D28" s="10">
         <f t="shared" si="1"/>
         <v>8.2500000000000004E-2</v>
       </c>
-      <c r="E28" s="11">
+      <c r="E28" s="10">
         <f t="shared" si="2"/>
         <v>0.11</v>
       </c>
-      <c r="F28" s="11">
+      <c r="F28" s="10">
         <f t="shared" si="1"/>
         <v>0.10400000000000001</v>
       </c>
-      <c r="G28" s="10">
+      <c r="G28" s="9">
         <f t="shared" si="3"/>
         <v>0.63301960784313727</v>
       </c>
@@ -1922,27 +2488,27 @@
       <c r="A29" t="s">
         <v>14</v>
       </c>
-      <c r="B29" s="11">
+      <c r="B29" s="10">
         <f t="shared" si="1"/>
         <v>0.22941176470588234</v>
       </c>
-      <c r="C29" s="11">
+      <c r="C29" s="10">
         <f t="shared" si="1"/>
         <v>0.17600000000000002</v>
       </c>
-      <c r="D29" s="11">
+      <c r="D29" s="10">
         <f t="shared" si="1"/>
         <v>0.11</v>
       </c>
-      <c r="E29" s="11">
+      <c r="E29" s="10">
         <f t="shared" si="2"/>
         <v>5.5E-2</v>
       </c>
-      <c r="F29" s="11">
+      <c r="F29" s="10">
         <f t="shared" si="1"/>
         <v>0.22533333333333333</v>
       </c>
-      <c r="G29" s="10">
+      <c r="G29" s="9">
         <f t="shared" si="3"/>
         <v>0.79574509803921578</v>
       </c>
@@ -1951,29 +2517,328 @@
       <c r="A30" t="s">
         <v>30</v>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="10">
         <f t="shared" si="1"/>
         <v>0.21666666666666667</v>
       </c>
-      <c r="C30" s="11">
+      <c r="C30" s="10">
         <f t="shared" si="1"/>
         <v>0.14799999999999999</v>
       </c>
-      <c r="D30" s="11">
+      <c r="D30" s="10">
         <f t="shared" si="1"/>
         <v>8.2500000000000004E-2</v>
       </c>
-      <c r="E30" s="11">
+      <c r="E30" s="10">
         <f t="shared" si="2"/>
         <v>3.793103448275862E-2</v>
       </c>
-      <c r="F30" s="11">
+      <c r="F30" s="10">
         <f t="shared" si="1"/>
         <v>0.2513333333333333</v>
       </c>
-      <c r="G30" s="10">
+      <c r="G30" s="9">
         <f t="shared" si="3"/>
         <v>0.73643103448275871</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="B33" t="s">
+        <v>50</v>
+      </c>
+      <c r="C33" t="s">
+        <v>51</v>
+      </c>
+      <c r="D33" t="s">
+        <v>52</v>
+      </c>
+      <c r="E33" t="s">
+        <v>53</v>
+      </c>
+      <c r="F33" t="s">
+        <v>54</v>
+      </c>
+      <c r="G33" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="B34" s="10">
+        <v>0.20392156862745098</v>
+      </c>
+      <c r="C34" s="10">
+        <v>0.22</v>
+      </c>
+      <c r="D34" s="10">
+        <v>8.2500000000000004E-2</v>
+      </c>
+      <c r="E34" s="10">
+        <v>4.5833333333333337E-2</v>
+      </c>
+      <c r="F34" s="10">
+        <v>0.26</v>
+      </c>
+      <c r="G34" s="9">
+        <v>0.81225490196078431</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="B35" s="10">
+        <v>0.26</v>
+      </c>
+      <c r="C35" s="10">
+        <v>0.26</v>
+      </c>
+      <c r="D35" s="10">
+        <v>5.5E-2</v>
+      </c>
+      <c r="E35" s="10">
+        <v>4.9999999999999996E-2</v>
+      </c>
+      <c r="F35" s="10">
+        <v>0.182</v>
+      </c>
+      <c r="G35" s="9">
+        <v>0.80700000000000016</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B36" s="10">
+        <v>0.22941176470588234</v>
+      </c>
+      <c r="C36" s="10">
+        <v>0.17600000000000002</v>
+      </c>
+      <c r="D36" s="10">
+        <v>0.11</v>
+      </c>
+      <c r="E36" s="10">
+        <v>5.5E-2</v>
+      </c>
+      <c r="F36" s="10">
+        <v>0.22533333333333333</v>
+      </c>
+      <c r="G36" s="9">
+        <v>0.79574509803921578</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="B37" s="10">
+        <v>0.21666666666666667</v>
+      </c>
+      <c r="C37" s="10">
+        <v>0.14799999999999999</v>
+      </c>
+      <c r="D37" s="10">
+        <v>8.2500000000000004E-2</v>
+      </c>
+      <c r="E37" s="10">
+        <v>3.793103448275862E-2</v>
+      </c>
+      <c r="F37" s="10">
+        <v>0.2513333333333333</v>
+      </c>
+      <c r="G37" s="9">
+        <v>0.73643103448275871</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A38" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B38" s="10">
+        <v>0.16887254901960785</v>
+      </c>
+      <c r="C38" s="10">
+        <v>0.252</v>
+      </c>
+      <c r="D38" s="10">
+        <v>8.2500000000000004E-2</v>
+      </c>
+      <c r="E38" s="10">
+        <v>6.1111111111111116E-2</v>
+      </c>
+      <c r="F38" s="10">
+        <v>0.16466666666666666</v>
+      </c>
+      <c r="G38" s="9">
+        <v>0.72915032679738556</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A39" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="B39" s="10">
+        <v>0.19754901960784313</v>
+      </c>
+      <c r="C39" s="10">
+        <v>0.21600000000000003</v>
+      </c>
+      <c r="D39" s="10">
+        <v>8.2500000000000004E-2</v>
+      </c>
+      <c r="E39" s="10">
+        <v>6.1111111111111116E-2</v>
+      </c>
+      <c r="F39" s="10">
+        <v>0.16466666666666666</v>
+      </c>
+      <c r="G39" s="9">
+        <v>0.72182679738562094</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A40" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="B40" s="10">
+        <v>0.21921568627450982</v>
+      </c>
+      <c r="C40" s="10">
+        <v>0.16</v>
+      </c>
+      <c r="D40" s="10">
+        <v>8.2500000000000004E-2</v>
+      </c>
+      <c r="E40" s="10">
+        <v>3.3846153846153845E-2</v>
+      </c>
+      <c r="F40" s="10">
+        <v>0.20800000000000002</v>
+      </c>
+      <c r="G40" s="9">
+        <v>0.70356184012066381</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A41" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B41" s="10">
+        <v>0.2077450980392157</v>
+      </c>
+      <c r="C41" s="10">
+        <v>0.17600000000000002</v>
+      </c>
+      <c r="D41" s="10">
+        <v>0.11</v>
+      </c>
+      <c r="E41" s="10">
+        <v>4.2307692307692303E-2</v>
+      </c>
+      <c r="F41" s="10">
+        <v>0.16466666666666666</v>
+      </c>
+      <c r="G41" s="9">
+        <v>0.70071945701357463</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A42" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="B42" s="10">
+        <v>0.20392156862745098</v>
+      </c>
+      <c r="C42" s="10">
+        <v>0.16</v>
+      </c>
+      <c r="D42" s="10">
+        <v>8.2500000000000004E-2</v>
+      </c>
+      <c r="E42" s="10">
+        <v>9.9999999999999992E-2</v>
+      </c>
+      <c r="F42" s="10">
+        <v>0.12133333333333333</v>
+      </c>
+      <c r="G42" s="9">
+        <v>0.66775490196078424</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A43" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="B43" s="10">
+        <v>0.16313725490196079</v>
+      </c>
+      <c r="C43" s="10">
+        <v>6.4000000000000001E-2</v>
+      </c>
+      <c r="D43" s="10">
+        <v>8.2500000000000004E-2</v>
+      </c>
+      <c r="E43" s="10">
+        <v>0.11</v>
+      </c>
+      <c r="F43" s="10">
+        <v>0.22533333333333333</v>
+      </c>
+      <c r="G43" s="9">
+        <v>0.64497058823529407</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A44" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="B44" s="10">
+        <v>0.17651960784313728</v>
+      </c>
+      <c r="C44" s="10">
+        <v>0.16</v>
+      </c>
+      <c r="D44" s="10">
+        <v>8.2500000000000004E-2</v>
+      </c>
+      <c r="E44" s="10">
+        <v>0.11</v>
+      </c>
+      <c r="F44" s="10">
+        <v>0.10400000000000001</v>
+      </c>
+      <c r="G44" s="9">
+        <v>0.63301960784313727</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A45" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="B45" s="10">
+        <v>0.17843137254901961</v>
+      </c>
+      <c r="C45" s="10">
+        <v>0.14799999999999999</v>
+      </c>
+      <c r="D45" s="10">
+        <v>0.11</v>
+      </c>
+      <c r="E45" s="10">
+        <v>5.5E-2</v>
+      </c>
+      <c r="F45" s="10">
+        <v>7.8E-2</v>
+      </c>
+      <c r="G45" s="9">
+        <v>0.56943137254901954</v>
       </c>
     </row>
   </sheetData>
@@ -1983,15 +2848,16 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63C902CE-5066-45BF-BEA2-646F8D396124}">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21" customWidth="1"/>
-    <col min="2" max="2" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.90625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="36.6328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="22.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="39.08984375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.26953125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.35">
@@ -2310,27 +3176,27 @@
       <c r="A17" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="10">
         <f>(B2/B$13)*B$14</f>
         <v>0.24555555555555555</v>
       </c>
-      <c r="C17" s="11">
+      <c r="C17" s="10">
         <f t="shared" ref="C17:F17" si="0">(C2/C$13)*C$14</f>
         <v>0.18255319148936172</v>
       </c>
-      <c r="D17" s="11">
+      <c r="D17" s="10">
         <f t="shared" si="0"/>
         <v>6.6000000000000003E-2</v>
       </c>
-      <c r="E17" s="11">
+      <c r="E17" s="10">
         <f>($E$13/E2)*$E$14</f>
         <v>2.5384615384615384E-2</v>
       </c>
-      <c r="F17" s="11">
+      <c r="F17" s="10">
         <f t="shared" si="0"/>
         <v>0.12000000000000001</v>
       </c>
-      <c r="G17" s="10">
+      <c r="G17" s="9">
         <f>SUM(B17:F17)</f>
         <v>0.6394933624295327</v>
       </c>
@@ -2339,27 +3205,27 @@
       <c r="A18" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="11">
+      <c r="B18" s="10">
         <f t="shared" ref="B18:F26" si="1">(B3/B$13)*B$14</f>
         <v>0.15744444444444444</v>
       </c>
-      <c r="C18" s="11">
+      <c r="C18" s="10">
         <f t="shared" si="1"/>
         <v>0.14936170212765959</v>
       </c>
-      <c r="D18" s="11">
+      <c r="D18" s="10">
         <f t="shared" si="1"/>
         <v>8.8000000000000009E-2</v>
       </c>
-      <c r="E18" s="11">
+      <c r="E18" s="10">
         <f t="shared" ref="E18:E26" si="2">($E$13/E3)*$E$14</f>
         <v>2.75E-2</v>
       </c>
-      <c r="F18" s="11">
+      <c r="F18" s="10">
         <f t="shared" si="1"/>
         <v>0.24000000000000002</v>
       </c>
-      <c r="G18" s="10">
+      <c r="G18" s="9">
         <f t="shared" ref="G18:G26" si="3">SUM(B18:F18)</f>
         <v>0.66230614657210407</v>
       </c>
@@ -2368,27 +3234,27 @@
       <c r="A19" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="11">
+      <c r="B19" s="10">
         <f t="shared" si="1"/>
         <v>0.18055555555555555</v>
       </c>
-      <c r="C19" s="11">
+      <c r="C19" s="10">
         <f t="shared" si="1"/>
         <v>0.18255319148936172</v>
       </c>
-      <c r="D19" s="11">
+      <c r="D19" s="10">
         <f t="shared" si="1"/>
         <v>8.8000000000000009E-2</v>
       </c>
-      <c r="E19" s="11">
+      <c r="E19" s="10">
         <f t="shared" si="2"/>
         <v>0.06</v>
       </c>
-      <c r="F19" s="11">
+      <c r="F19" s="10">
         <f t="shared" si="1"/>
         <v>0.2</v>
       </c>
-      <c r="G19" s="10">
+      <c r="G19" s="9">
         <f t="shared" si="3"/>
         <v>0.71110874704491733</v>
       </c>
@@ -2397,27 +3263,27 @@
       <c r="A20" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="10">
         <f t="shared" si="1"/>
         <v>0.23544444444444446</v>
       </c>
-      <c r="C20" s="11">
+      <c r="C20" s="10">
         <f t="shared" si="1"/>
         <v>0.19914893617021276</v>
       </c>
-      <c r="D20" s="11">
+      <c r="D20" s="10">
         <f t="shared" si="1"/>
         <v>8.8000000000000009E-2</v>
       </c>
-      <c r="E20" s="11">
+      <c r="E20" s="10">
         <f t="shared" si="2"/>
         <v>2.5384615384615384E-2</v>
       </c>
-      <c r="F20" s="11">
+      <c r="F20" s="10">
         <f t="shared" si="1"/>
         <v>0.15000000000000002</v>
       </c>
-      <c r="G20" s="10">
+      <c r="G20" s="9">
         <f t="shared" si="3"/>
         <v>0.69797799599927257</v>
       </c>
@@ -2426,27 +3292,27 @@
       <c r="A21" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="10">
         <f t="shared" si="1"/>
         <v>0.15166666666666667</v>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="10">
         <f t="shared" si="1"/>
         <v>8.851063829787234E-2</v>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="10">
         <f t="shared" si="1"/>
         <v>8.8000000000000009E-2</v>
       </c>
-      <c r="E21" s="11">
+      <c r="E21" s="10">
         <f t="shared" si="2"/>
         <v>0.11</v>
       </c>
-      <c r="F21" s="11">
+      <c r="F21" s="10">
         <f t="shared" si="1"/>
         <v>0.13</v>
       </c>
-      <c r="G21" s="10">
+      <c r="G21" s="9">
         <f t="shared" si="3"/>
         <v>0.568177304964539</v>
       </c>
@@ -2455,27 +3321,27 @@
       <c r="A22" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="11">
+      <c r="B22" s="10">
         <f t="shared" si="1"/>
         <v>0.24555555555555555</v>
       </c>
-      <c r="C22" s="11">
+      <c r="C22" s="10">
         <f t="shared" si="1"/>
         <v>0.1327659574468085</v>
       </c>
-      <c r="D22" s="11">
+      <c r="D22" s="10">
         <f t="shared" si="1"/>
         <v>8.8000000000000009E-2</v>
       </c>
-      <c r="E22" s="11">
+      <c r="E22" s="10">
         <f t="shared" si="2"/>
         <v>0.03</v>
       </c>
-      <c r="F22" s="11">
+      <c r="F22" s="10">
         <f t="shared" si="1"/>
         <v>0.15000000000000002</v>
       </c>
-      <c r="G22" s="10">
+      <c r="G22" s="9">
         <f t="shared" si="3"/>
         <v>0.64632151300236407</v>
       </c>
@@ -2484,27 +3350,27 @@
       <c r="A23" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="11">
+      <c r="B23" s="10">
         <f t="shared" si="1"/>
         <v>0.1783888888888889</v>
       </c>
-      <c r="C23" s="11">
+      <c r="C23" s="10">
         <f t="shared" si="1"/>
         <v>0.14382978723404255</v>
       </c>
-      <c r="D23" s="11">
+      <c r="D23" s="10">
         <f t="shared" si="1"/>
         <v>6.6000000000000003E-2</v>
       </c>
-      <c r="E23" s="11">
+      <c r="E23" s="10">
         <f t="shared" si="2"/>
         <v>7.3333333333333334E-2</v>
       </c>
-      <c r="F23" s="11">
+      <c r="F23" s="10">
         <f t="shared" si="1"/>
         <v>0.17000000000000004</v>
       </c>
-      <c r="G23" s="10">
+      <c r="G23" s="9">
         <f t="shared" si="3"/>
         <v>0.63155200945626477</v>
       </c>
@@ -2513,27 +3379,27 @@
       <c r="A24" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="11">
+      <c r="B24" s="10">
         <f t="shared" si="1"/>
         <v>0.21594444444444447</v>
       </c>
-      <c r="C24" s="11">
+      <c r="C24" s="10">
         <f t="shared" si="1"/>
         <v>0.17702127659574468</v>
       </c>
-      <c r="D24" s="11">
+      <c r="D24" s="10">
         <f t="shared" si="1"/>
         <v>0.11</v>
       </c>
-      <c r="E24" s="11">
+      <c r="E24" s="10">
         <f t="shared" si="2"/>
         <v>5.0769230769230768E-2</v>
       </c>
-      <c r="F24" s="11">
+      <c r="F24" s="10">
         <f t="shared" si="1"/>
         <v>0.25000000000000006</v>
       </c>
-      <c r="G24" s="10">
+      <c r="G24" s="9">
         <f t="shared" si="3"/>
         <v>0.8037349518094199</v>
       </c>
@@ -2542,58 +3408,311 @@
       <c r="A25" t="s">
         <v>33</v>
       </c>
-      <c r="B25" s="11">
+      <c r="B25" s="10">
         <f t="shared" si="1"/>
         <v>0.23833333333333334</v>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="10">
         <f t="shared" si="1"/>
         <v>0.16042553191489362</v>
       </c>
-      <c r="D25" s="11">
+      <c r="D25" s="10">
         <f t="shared" si="1"/>
         <v>8.8000000000000009E-2</v>
       </c>
-      <c r="E25" s="11">
+      <c r="E25" s="10">
         <f t="shared" si="2"/>
         <v>0.06</v>
       </c>
-      <c r="F25" s="11">
+      <c r="F25" s="10">
         <f t="shared" si="1"/>
         <v>0.26</v>
       </c>
-      <c r="G25" s="10">
+      <c r="G25" s="9">
         <f t="shared" si="3"/>
         <v>0.80675886524822693</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" s="13" t="s">
+      <c r="A26" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="14">
+      <c r="B26" s="13">
         <f t="shared" si="1"/>
         <v>0.26</v>
       </c>
-      <c r="C26" s="14">
+      <c r="C26" s="13">
         <f t="shared" si="1"/>
         <v>0.26</v>
       </c>
-      <c r="D26" s="14">
+      <c r="D26" s="13">
         <f t="shared" si="1"/>
         <v>6.6000000000000003E-2</v>
       </c>
-      <c r="E26" s="14">
+      <c r="E26" s="13">
         <f t="shared" si="2"/>
         <v>7.3333333333333334E-2</v>
       </c>
-      <c r="F26" s="14">
+      <c r="F26" s="13">
         <f t="shared" si="1"/>
         <v>0.19000000000000003</v>
       </c>
-      <c r="G26" s="12">
+      <c r="G26" s="11">
         <f t="shared" si="3"/>
         <v>0.8493333333333335</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A29" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B29" t="s">
+        <v>50</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29" t="s">
+        <v>52</v>
+      </c>
+      <c r="E29" t="s">
+        <v>53</v>
+      </c>
+      <c r="F29" t="s">
+        <v>54</v>
+      </c>
+      <c r="G29" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A30" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="B30" s="10">
+        <v>0.26</v>
+      </c>
+      <c r="C30" s="10">
+        <v>0.26</v>
+      </c>
+      <c r="D30" s="10">
+        <v>6.6000000000000003E-2</v>
+      </c>
+      <c r="E30" s="10">
+        <v>7.3333333333333334E-2</v>
+      </c>
+      <c r="F30" s="10">
+        <v>0.19000000000000003</v>
+      </c>
+      <c r="G30" s="9">
+        <v>0.8493333333333335</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A31" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="10">
+        <v>0.23833333333333334</v>
+      </c>
+      <c r="C31" s="10">
+        <v>0.16042553191489362</v>
+      </c>
+      <c r="D31" s="10">
+        <v>8.8000000000000009E-2</v>
+      </c>
+      <c r="E31" s="10">
+        <v>0.06</v>
+      </c>
+      <c r="F31" s="10">
+        <v>0.26</v>
+      </c>
+      <c r="G31" s="9">
+        <v>0.80675886524822693</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A32" s="15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B32" s="10">
+        <v>0.21594444444444447</v>
+      </c>
+      <c r="C32" s="10">
+        <v>0.17702127659574468</v>
+      </c>
+      <c r="D32" s="10">
+        <v>0.11</v>
+      </c>
+      <c r="E32" s="10">
+        <v>5.0769230769230768E-2</v>
+      </c>
+      <c r="F32" s="10">
+        <v>0.25000000000000006</v>
+      </c>
+      <c r="G32" s="9">
+        <v>0.8037349518094199</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A33" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="B33" s="10">
+        <v>0.18055555555555555</v>
+      </c>
+      <c r="C33" s="10">
+        <v>0.18255319148936172</v>
+      </c>
+      <c r="D33" s="10">
+        <v>8.8000000000000009E-2</v>
+      </c>
+      <c r="E33" s="10">
+        <v>0.06</v>
+      </c>
+      <c r="F33" s="10">
+        <v>0.2</v>
+      </c>
+      <c r="G33" s="9">
+        <v>0.71110874704491733</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A34" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B34" s="10">
+        <v>0.23544444444444446</v>
+      </c>
+      <c r="C34" s="10">
+        <v>0.19914893617021276</v>
+      </c>
+      <c r="D34" s="10">
+        <v>8.8000000000000009E-2</v>
+      </c>
+      <c r="E34" s="10">
+        <v>2.5384615384615384E-2</v>
+      </c>
+      <c r="F34" s="10">
+        <v>0.15000000000000002</v>
+      </c>
+      <c r="G34" s="9">
+        <v>0.69797799599927257</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A35" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B35" s="10">
+        <v>0.15744444444444444</v>
+      </c>
+      <c r="C35" s="10">
+        <v>0.14936170212765959</v>
+      </c>
+      <c r="D35" s="10">
+        <v>8.8000000000000009E-2</v>
+      </c>
+      <c r="E35" s="10">
+        <v>2.75E-2</v>
+      </c>
+      <c r="F35" s="10">
+        <v>0.24000000000000002</v>
+      </c>
+      <c r="G35" s="9">
+        <v>0.66230614657210407</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A36" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B36" s="10">
+        <v>0.24555555555555555</v>
+      </c>
+      <c r="C36" s="10">
+        <v>0.1327659574468085</v>
+      </c>
+      <c r="D36" s="10">
+        <v>8.8000000000000009E-2</v>
+      </c>
+      <c r="E36" s="10">
+        <v>0.03</v>
+      </c>
+      <c r="F36" s="10">
+        <v>0.15000000000000002</v>
+      </c>
+      <c r="G36" s="9">
+        <v>0.64632151300236407</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A37" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B37" s="10">
+        <v>0.24555555555555555</v>
+      </c>
+      <c r="C37" s="10">
+        <v>0.18255319148936172</v>
+      </c>
+      <c r="D37" s="10">
+        <v>6.6000000000000003E-2</v>
+      </c>
+      <c r="E37" s="10">
+        <v>2.5384615384615384E-2</v>
+      </c>
+      <c r="F37" s="10">
+        <v>0.12000000000000001</v>
+      </c>
+      <c r="G37" s="9">
+        <v>0.6394933624295327</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A38" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B38" s="10">
+        <v>0.1783888888888889</v>
+      </c>
+      <c r="C38" s="10">
+        <v>0.14382978723404255</v>
+      </c>
+      <c r="D38" s="10">
+        <v>6.6000000000000003E-2</v>
+      </c>
+      <c r="E38" s="10">
+        <v>7.3333333333333334E-2</v>
+      </c>
+      <c r="F38" s="10">
+        <v>0.17000000000000004</v>
+      </c>
+      <c r="G38" s="9">
+        <v>0.63155200945626477</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="A39" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="B39" s="10">
+        <v>0.15166666666666667</v>
+      </c>
+      <c r="C39" s="10">
+        <v>8.851063829787234E-2</v>
+      </c>
+      <c r="D39" s="10">
+        <v>8.8000000000000009E-2</v>
+      </c>
+      <c r="E39" s="10">
+        <v>0.11</v>
+      </c>
+      <c r="F39" s="10">
+        <v>0.13</v>
+      </c>
+      <c r="G39" s="9">
+        <v>0.568177304964539</v>
       </c>
     </row>
   </sheetData>

</xml_diff>